<commit_message>
done mapped headers - wl report
</commit_message>
<xml_diff>
--- a/needs/wl needs/template dump.xlsx
+++ b/needs/wl needs/template dump.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SOLIZA\Documents\secret\needs\wl needs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92CF7D09-0F5A-4C5B-A287-49D9674F6364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C1C9294-1C82-45B0-A237-99D20A7132F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{4AB12ACA-EEE0-4203-AAF1-F3759D1CA7C3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="102">
   <si>
     <t>CUST_ID</t>
   </si>
@@ -339,6 +339,9 @@
   </si>
   <si>
     <t>TEMPLATE</t>
+  </si>
+  <si>
+    <t>DATE</t>
   </si>
 </sst>
 </file>
@@ -433,8 +436,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -797,10 +799,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B07FC59E-C563-4BBF-A014-E6B0170ADE0A}">
-  <dimension ref="A1:AS10"/>
+  <dimension ref="A1:AS18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
@@ -846,840 +848,870 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
-      <c r="X1" s="3" t="s">
+      <c r="V1" s="4"/>
+      <c r="W1" s="4"/>
+      <c r="X1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Y1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AA1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AB1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AD1" s="5"/>
-      <c r="AE1" s="5"/>
-      <c r="AF1" s="5"/>
-      <c r="AG1" s="5"/>
-      <c r="AH1" s="5"/>
-      <c r="AI1" s="5"/>
-      <c r="AJ1" s="5"/>
-      <c r="AK1" s="5"/>
-      <c r="AL1" s="5"/>
-      <c r="AM1" s="5"/>
-      <c r="AN1" s="5"/>
-      <c r="AO1" s="5"/>
-      <c r="AP1" s="5"/>
-      <c r="AQ1" s="5"/>
-      <c r="AR1" s="5"/>
-      <c r="AS1" s="5"/>
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
+      <c r="AH1" s="4"/>
+      <c r="AI1" s="4"/>
+      <c r="AJ1" s="4"/>
+      <c r="AK1" s="4"/>
+      <c r="AL1" s="4"/>
+      <c r="AM1" s="4"/>
+      <c r="AN1" s="4"/>
+      <c r="AO1" s="4"/>
+      <c r="AP1" s="4"/>
+      <c r="AQ1" s="4"/>
+      <c r="AR1" s="4"/>
+      <c r="AS1" s="4"/>
     </row>
     <row r="2" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="P2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="Q2" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="R2" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="6" t="s">
+      <c r="S2" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="T2" s="6" t="s">
+      <c r="T2" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="U2" s="6" t="s">
+      <c r="U2" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="V2" s="6" t="s">
+      <c r="V2" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="W2" s="6" t="s">
+      <c r="W2" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="X2" s="6" t="s">
+      <c r="X2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="Y2" s="6" t="s">
+      <c r="Y2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="Z2" s="6" t="s">
+      <c r="Z2" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="AA2" s="6" t="s">
+      <c r="AA2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AB2" s="6" t="s">
+      <c r="AB2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="AC2" s="6" t="s">
+      <c r="AC2" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AD2" s="5"/>
-      <c r="AE2" s="5"/>
-      <c r="AF2" s="5"/>
-      <c r="AG2" s="5"/>
-      <c r="AH2" s="5"/>
-      <c r="AI2" s="5"/>
-      <c r="AJ2" s="5"/>
-      <c r="AK2" s="5"/>
-      <c r="AL2" s="5"/>
-      <c r="AM2" s="5"/>
-      <c r="AN2" s="5"/>
-      <c r="AO2" s="5"/>
-      <c r="AP2" s="5"/>
-      <c r="AQ2" s="5"/>
-      <c r="AR2" s="5"/>
-      <c r="AS2" s="5"/>
+      <c r="AD2" s="4"/>
+      <c r="AE2" s="4"/>
+      <c r="AF2" s="4"/>
+      <c r="AG2" s="4"/>
+      <c r="AH2" s="4"/>
+      <c r="AI2" s="4"/>
+      <c r="AJ2" s="4"/>
+      <c r="AK2" s="4"/>
+      <c r="AL2" s="4"/>
+      <c r="AM2" s="4"/>
+      <c r="AN2" s="4"/>
+      <c r="AO2" s="4"/>
+      <c r="AP2" s="4"/>
+      <c r="AQ2" s="4"/>
+      <c r="AR2" s="4"/>
+      <c r="AS2" s="4"/>
     </row>
     <row r="3" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="5">
         <v>508518.17</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="5">
         <v>508518.17</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="L3" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="M3" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3" s="5">
         <v>12821.88</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="O3" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="P3" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="Q3" s="6" t="s">
+      <c r="Q3" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="R3" s="6" t="s">
+      <c r="R3" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="S3" s="7">
+      <c r="S3" s="6">
         <v>1</v>
       </c>
-      <c r="T3" s="6" t="s">
+      <c r="T3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="U3" s="6" t="s">
+      <c r="U3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="V3" s="6" t="s">
+      <c r="V3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="W3" s="6" t="s">
+      <c r="W3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="X3" s="6" t="s">
+      <c r="X3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="Y3" s="7">
+      <c r="Y3" s="6">
         <v>46097</v>
       </c>
-      <c r="Z3" s="6" t="s">
+      <c r="Z3" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="AA3" s="6" t="s">
+      <c r="AA3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="AB3" s="7">
+      <c r="AB3" s="6">
         <v>34298</v>
       </c>
-      <c r="AC3" s="6" t="s">
+      <c r="AC3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="AD3" s="5"/>
-      <c r="AE3" s="5"/>
-      <c r="AF3" s="5"/>
-      <c r="AG3" s="5"/>
-      <c r="AH3" s="5"/>
-      <c r="AI3" s="5"/>
-      <c r="AJ3" s="5"/>
-      <c r="AK3" s="5"/>
-      <c r="AL3" s="5"/>
-      <c r="AM3" s="5"/>
-      <c r="AN3" s="5"/>
-      <c r="AO3" s="5"/>
-      <c r="AP3" s="5"/>
-      <c r="AQ3" s="5"/>
-      <c r="AR3" s="5"/>
-      <c r="AS3" s="5"/>
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4"/>
+      <c r="AF3" s="4"/>
+      <c r="AG3" s="4"/>
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4"/>
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="4"/>
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4"/>
+      <c r="AN3" s="4"/>
+      <c r="AO3" s="4"/>
+      <c r="AP3" s="4"/>
+      <c r="AQ3" s="4"/>
+      <c r="AR3" s="4"/>
+      <c r="AS3" s="4"/>
     </row>
-    <row r="4" spans="1:45" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>242809.73</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="5">
         <v>242809.73</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="5">
         <v>16178.01</v>
       </c>
-      <c r="O4" s="6" t="s">
+      <c r="O4" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="P4" s="6" t="s">
+      <c r="P4" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="Q4" s="6" t="s">
+      <c r="Q4" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="R4" s="6" t="s">
+      <c r="R4" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="S4" s="7">
+      <c r="S4" s="6">
         <v>28454</v>
       </c>
-      <c r="T4" s="6">
+      <c r="T4" s="5">
         <v>46122</v>
       </c>
-      <c r="U4" s="6">
+      <c r="U4" s="5">
         <v>8210</v>
       </c>
-      <c r="V4" s="6" t="s">
+      <c r="V4" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="W4" s="6" t="s">
+      <c r="W4" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="X4" s="6" t="s">
+      <c r="X4" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="Y4" s="7">
+      <c r="Y4" s="6">
         <v>46097</v>
       </c>
-      <c r="Z4" s="6" t="s">
+      <c r="Z4" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="AA4" s="6" t="s">
+      <c r="AA4" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="7">
+      <c r="AB4" s="6">
         <v>41197</v>
       </c>
-      <c r="AC4" s="6" t="s">
+      <c r="AC4" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="AD4" s="5"/>
-      <c r="AE4" s="5"/>
-      <c r="AF4" s="5"/>
-      <c r="AG4" s="5"/>
-      <c r="AH4" s="5"/>
-      <c r="AI4" s="5"/>
-      <c r="AJ4" s="5"/>
-      <c r="AK4" s="5"/>
-      <c r="AL4" s="5"/>
-      <c r="AM4" s="5"/>
-      <c r="AN4" s="5"/>
-      <c r="AO4" s="5"/>
-      <c r="AP4" s="5"/>
-      <c r="AQ4" s="5"/>
-      <c r="AR4" s="5"/>
-      <c r="AS4" s="5"/>
+      <c r="AD4" s="4"/>
+      <c r="AE4" s="4"/>
+      <c r="AF4" s="4"/>
+      <c r="AG4" s="4"/>
+      <c r="AH4" s="4"/>
+      <c r="AI4" s="4"/>
+      <c r="AJ4" s="4"/>
+      <c r="AK4" s="4"/>
+      <c r="AL4" s="4"/>
+      <c r="AM4" s="4"/>
+      <c r="AN4" s="4"/>
+      <c r="AO4" s="4"/>
+      <c r="AP4" s="4"/>
+      <c r="AQ4" s="4"/>
+      <c r="AR4" s="4"/>
+      <c r="AS4" s="4"/>
     </row>
     <row r="5" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O5" s="3" t="s">
+      <c r="O5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P5" s="3" t="s">
+      <c r="P5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="3" t="s">
+      <c r="Q5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R5" s="3" t="s">
+      <c r="R5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S5" s="2" t="s">
+      <c r="S5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T5" s="2" t="s">
+      <c r="T5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U5" s="2" t="s">
+      <c r="U5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V5" s="3" t="s">
+      <c r="V5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W5" s="3" t="s">
+      <c r="W5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X5" s="3" t="s">
+      <c r="X5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y5" s="3" t="s">
+      <c r="Y5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z5" s="3" t="s">
+      <c r="Z5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA5" s="4" t="s">
+      <c r="AA5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AB5" s="2" t="s">
+      <c r="AB5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC5" s="2" t="s">
+      <c r="AC5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD5" s="3" t="s">
+      <c r="AD5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE5" s="4" t="s">
+      <c r="AE5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AF5" s="3" t="s">
+      <c r="AF5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG5" s="4" t="s">
+      <c r="AG5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AH5" s="3" t="s">
+      <c r="AH5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI5" s="2" t="s">
+      <c r="AI5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ5" s="3" t="s">
+      <c r="AJ5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK5" s="3" t="s">
+      <c r="AK5" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL5" s="3" t="s">
+      <c r="AL5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM5" s="4" t="s">
+      <c r="AM5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="AN5" s="3" t="s">
+      <c r="AN5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AO5" s="2" t="s">
+      <c r="AO5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP5" s="2" t="s">
+      <c r="AP5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ5" s="2" t="s">
+      <c r="AQ5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR5" s="4" t="s">
+      <c r="AR5" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AS5" s="4" t="s">
+      <c r="AS5" s="3" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="8" t="s">
+      <c r="F6" s="8"/>
+      <c r="G6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="8">
+      <c r="H6" s="8"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="7">
         <v>508518.17</v>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="7">
         <v>508518.17</v>
       </c>
-      <c r="N6" s="8">
+      <c r="N6" s="7">
         <v>521340.05</v>
       </c>
-      <c r="O6" s="8">
+      <c r="O6" s="7">
         <v>31878.04</v>
       </c>
-      <c r="P6" s="8">
+      <c r="P6" s="7">
         <v>13258.75</v>
       </c>
-      <c r="Q6" s="8">
+      <c r="Q6" s="7">
         <v>12821.88</v>
       </c>
-      <c r="R6" s="8" t="s">
+      <c r="R6" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="S6" s="9"/>
-      <c r="T6" s="9"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="8" t="s">
+      <c r="S6" s="8"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="W6" s="8" t="s">
+      <c r="W6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="X6" s="8" t="s">
+      <c r="X6" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="Y6" s="8" t="s">
+      <c r="Y6" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="Z6" s="8" t="s">
+      <c r="Z6" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="AA6" s="10"/>
-      <c r="AB6" s="9"/>
-      <c r="AC6" s="9"/>
-      <c r="AD6" s="8"/>
-      <c r="AE6" s="10"/>
-      <c r="AF6" s="8" t="s">
+      <c r="AA6" s="9"/>
+      <c r="AB6" s="8"/>
+      <c r="AC6" s="8"/>
+      <c r="AD6" s="7"/>
+      <c r="AE6" s="9"/>
+      <c r="AF6" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="AG6" s="10"/>
-      <c r="AH6" s="8"/>
-      <c r="AI6" s="9"/>
-      <c r="AJ6" s="8" t="s">
+      <c r="AG6" s="9"/>
+      <c r="AH6" s="7"/>
+      <c r="AI6" s="8"/>
+      <c r="AJ6" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AK6" s="8" t="s">
+      <c r="AK6" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="AL6" s="8"/>
-      <c r="AM6" s="10"/>
-      <c r="AN6" s="8" t="s">
+      <c r="AL6" s="7"/>
+      <c r="AM6" s="9"/>
+      <c r="AN6" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="AO6" s="9"/>
-      <c r="AP6" s="9"/>
-      <c r="AQ6" s="9"/>
-      <c r="AR6" s="10"/>
-      <c r="AS6" s="10"/>
+      <c r="AO6" s="8"/>
+      <c r="AP6" s="8"/>
+      <c r="AQ6" s="8"/>
+      <c r="AR6" s="9"/>
+      <c r="AS6" s="9"/>
     </row>
-    <row r="7" spans="1:45" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+    <row r="7" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="8" t="s">
+      <c r="F7" s="8"/>
+      <c r="G7" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="8" t="s">
+      <c r="H7" s="8"/>
+      <c r="I7" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="8">
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="7">
         <v>242809.73</v>
       </c>
-      <c r="M7" s="8">
+      <c r="M7" s="7">
         <v>242809.73</v>
       </c>
-      <c r="N7" s="8">
+      <c r="N7" s="7">
         <v>242809.73</v>
       </c>
-      <c r="O7" s="8">
+      <c r="O7" s="7">
         <v>16881.54</v>
       </c>
-      <c r="P7" s="8">
+      <c r="P7" s="7">
         <v>8209.76</v>
       </c>
-      <c r="Q7" s="8">
+      <c r="Q7" s="7">
         <v>16178.01</v>
       </c>
-      <c r="R7" s="8" t="s">
+      <c r="R7" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="S7" s="9"/>
-      <c r="T7" s="9"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="8" t="s">
+      <c r="S7" s="8"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="8"/>
+      <c r="V7" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="W7" s="8" t="s">
+      <c r="W7" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="X7" s="8" t="s">
+      <c r="X7" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="Y7" s="8" t="s">
+      <c r="Y7" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="Z7" s="8" t="s">
+      <c r="Z7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="AA7" s="10" t="s">
+      <c r="AA7" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="AB7" s="9"/>
-      <c r="AC7" s="9"/>
-      <c r="AD7" s="8"/>
-      <c r="AE7" s="10"/>
-      <c r="AF7" s="8" t="s">
+      <c r="AB7" s="8"/>
+      <c r="AC7" s="8"/>
+      <c r="AD7" s="7"/>
+      <c r="AE7" s="9"/>
+      <c r="AF7" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="AG7" s="10"/>
-      <c r="AH7" s="8"/>
-      <c r="AI7" s="9"/>
-      <c r="AJ7" s="8" t="s">
+      <c r="AG7" s="9"/>
+      <c r="AH7" s="7"/>
+      <c r="AI7" s="8"/>
+      <c r="AJ7" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AK7" s="8" t="s">
+      <c r="AK7" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="AL7" s="8"/>
-      <c r="AM7" s="10"/>
-      <c r="AN7" s="8" t="s">
+      <c r="AL7" s="7"/>
+      <c r="AM7" s="9"/>
+      <c r="AN7" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="AO7" s="9"/>
-      <c r="AP7" s="9"/>
-      <c r="AQ7" s="9"/>
-      <c r="AR7" s="10"/>
-      <c r="AS7" s="10"/>
+      <c r="AO7" s="8"/>
+      <c r="AP7" s="8"/>
+      <c r="AQ7" s="8"/>
+      <c r="AR7" s="9"/>
+      <c r="AS7" s="9"/>
     </row>
     <row r="8" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="5"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="5"/>
-      <c r="T8" s="5"/>
-      <c r="U8" s="5"/>
-      <c r="V8" s="5"/>
-      <c r="W8" s="5"/>
-      <c r="X8" s="5"/>
-      <c r="Y8" s="5"/>
-      <c r="Z8" s="5"/>
-      <c r="AA8" s="5"/>
-      <c r="AB8" s="5"/>
-      <c r="AC8" s="5"/>
-      <c r="AD8" s="5"/>
-      <c r="AE8" s="5"/>
-      <c r="AF8" s="5"/>
-      <c r="AG8" s="5"/>
-      <c r="AH8" s="5"/>
-      <c r="AI8" s="5"/>
-      <c r="AJ8" s="5"/>
-      <c r="AK8" s="5"/>
-      <c r="AL8" s="5"/>
-      <c r="AM8" s="5"/>
-      <c r="AN8" s="5"/>
-      <c r="AO8" s="5"/>
-      <c r="AP8" s="5"/>
-      <c r="AQ8" s="5"/>
-      <c r="AR8" s="5"/>
-      <c r="AS8" s="5"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
+      <c r="W8" s="4"/>
+      <c r="X8" s="4"/>
+      <c r="Y8" s="4"/>
+      <c r="Z8" s="4"/>
+      <c r="AA8" s="4"/>
+      <c r="AB8" s="4"/>
+      <c r="AC8" s="4"/>
+      <c r="AD8" s="4"/>
+      <c r="AE8" s="4"/>
+      <c r="AF8" s="4"/>
+      <c r="AG8" s="4"/>
+      <c r="AH8" s="4"/>
+      <c r="AI8" s="4"/>
+      <c r="AJ8" s="4"/>
+      <c r="AK8" s="4"/>
+      <c r="AL8" s="4"/>
+      <c r="AM8" s="4"/>
+      <c r="AN8" s="4"/>
+      <c r="AO8" s="4"/>
+      <c r="AP8" s="4"/>
+      <c r="AQ8" s="4"/>
+      <c r="AR8" s="4"/>
+      <c r="AS8" s="4"/>
     </row>
     <row r="9" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="5"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="5"/>
-      <c r="T9" s="5"/>
-      <c r="U9" s="5"/>
-      <c r="V9" s="5"/>
-      <c r="W9" s="5"/>
-      <c r="X9" s="5"/>
-      <c r="Y9" s="5"/>
-      <c r="Z9" s="5"/>
-      <c r="AA9" s="5"/>
-      <c r="AB9" s="5"/>
-      <c r="AC9" s="5"/>
-      <c r="AD9" s="5"/>
-      <c r="AE9" s="5"/>
-      <c r="AF9" s="5"/>
-      <c r="AG9" s="5"/>
-      <c r="AH9" s="5"/>
-      <c r="AI9" s="5"/>
-      <c r="AJ9" s="5"/>
-      <c r="AK9" s="5"/>
-      <c r="AL9" s="5"/>
-      <c r="AM9" s="5"/>
-      <c r="AN9" s="5"/>
-      <c r="AO9" s="5"/>
-      <c r="AP9" s="5"/>
-      <c r="AQ9" s="5"/>
-      <c r="AR9" s="5"/>
-      <c r="AS9" s="5"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
+      <c r="W9" s="4"/>
+      <c r="X9" s="4"/>
+      <c r="Y9" s="4"/>
+      <c r="Z9" s="4"/>
+      <c r="AA9" s="4"/>
+      <c r="AB9" s="4"/>
+      <c r="AC9" s="4"/>
+      <c r="AD9" s="4"/>
+      <c r="AE9" s="4"/>
+      <c r="AF9" s="4"/>
+      <c r="AG9" s="4"/>
+      <c r="AH9" s="4"/>
+      <c r="AI9" s="4"/>
+      <c r="AJ9" s="4"/>
+      <c r="AK9" s="4"/>
+      <c r="AL9" s="4"/>
+      <c r="AM9" s="4"/>
+      <c r="AN9" s="4"/>
+      <c r="AO9" s="4"/>
+      <c r="AP9" s="4"/>
+      <c r="AQ9" s="4"/>
+      <c r="AR9" s="4"/>
+      <c r="AS9" s="4"/>
     </row>
     <row r="10" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>